<commit_message>
feat: implement heatmap working with new format
</commit_message>
<xml_diff>
--- a/files/muscle-categorization.xlsx
+++ b/files/muscle-categorization.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Job\fitcode\fitcode\files\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4B8A0264-2E41-4D13-9E99-29E172E7FE67}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{23185212-49DE-4896-8DB4-D8C2406C401F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-11805" yWindow="-21720" windowWidth="51840" windowHeight="21120" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="553" uniqueCount="165">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1112" uniqueCount="167">
   <si>
     <t>trapezius-r</t>
   </si>
@@ -523,6 +523,12 @@
   </si>
   <si>
     <t>MUSCLE (LEVEL 4)</t>
+  </si>
+  <si>
+    <t>Latisimus Dorsi</t>
+  </si>
+  <si>
+    <t>Serratus Posterior</t>
   </si>
 </sst>
 </file>
@@ -2212,7 +2218,9 @@
       <c r="A93" s="3" t="s">
         <v>89</v>
       </c>
-      <c r="B93" s="3"/>
+      <c r="B93" s="3" t="s">
+        <v>165</v>
+      </c>
       <c r="C93" t="s">
         <v>156</v>
       </c>
@@ -2224,7 +2232,9 @@
       <c r="A94" s="3" t="s">
         <v>90</v>
       </c>
-      <c r="B94" s="3"/>
+      <c r="B94" s="3" t="s">
+        <v>165</v>
+      </c>
       <c r="C94" t="s">
         <v>156</v>
       </c>
@@ -2432,7 +2442,9 @@
       <c r="A109" t="s">
         <v>101</v>
       </c>
-      <c r="B109" s="3"/>
+      <c r="B109" s="3" t="s">
+        <v>166</v>
+      </c>
       <c r="C109" t="s">
         <v>155</v>
       </c>

</xml_diff>